<commit_message>
Update published master datasets (2026-10-14)
</commit_message>
<xml_diff>
--- a/outputs/InnovateUK_Funding_Opportunities_Latest.xlsx
+++ b/outputs/InnovateUK_Funding_Opportunities_Latest.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -503,26 +503,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Innovate Funding Service</t>
+          <t>Innovate UK Business Connect</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BridgeAI Deployment Catalyst: AI for Assurance and Compliance</t>
+          <t>HMGCC Co-Creation Challenge: Multi-Terrain Micro Robotic Systems</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2597/overview/7ec02a95-73e5-4928-8104-67a9f1b279e3</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/hmgcc-co-creation-challenge-multi-terrain-micro-robotic-systems/</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-06 16:27</t>
+          <t>2026-10-12 19:27</t>
         </is>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46301.68541666667</v>
+        <v>46307.81041666667</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
@@ -531,48 +531,52 @@
       <c r="H2" t="b">
         <v>0</v>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+      <c r="J2" s="1" t="n">
+        <v>46307</v>
+      </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Tuesday 8 December 2026 11:00am</t>
-        </is>
-      </c>
-      <c r="L2" s="1" t="n">
-        <v>46364.45833333334</v>
-      </c>
+          <t>12/11/2026</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>£200,000</t>
+          <t>£60,000</t>
         </is>
       </c>
       <c r="N2" s="1" t="n">
-        <v>46295</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Innovate Funding Service</t>
+          <t>Innovate UK Business Connect</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BridgeAI Deployment Catalyst: AI for Decision Critical Systems</t>
+          <t>HMGCC Co-Creation Challenge: Smart glasses for mapping</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2598/overview/cfb35198-55fc-4aad-afa1-86a260bfaddf</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/hmgcc-co-creation-challenge-smart-glasses-for-mapping/</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-06 16:27</t>
+          <t>2026-10-12 19:27</t>
         </is>
       </c>
       <c r="E3" s="1" t="n">
-        <v>46301.68541666667</v>
+        <v>46307.81041666667</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
@@ -581,29 +585,33 @@
       <c r="H3" t="b">
         <v>0</v>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+      <c r="J3" s="1" t="n">
+        <v>46307</v>
+      </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Tuesday 8 December 2026 11:00am</t>
-        </is>
-      </c>
-      <c r="L3" s="1" t="n">
-        <v>46364.45833333334</v>
-      </c>
+          <t>12/11/2026</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>£200,000</t>
+          <t>£60,000</t>
         </is>
       </c>
       <c r="N3" s="1" t="n">
-        <v>46295</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Innovate Funding Service</t>
+          <t>Innovate UK Business Connect</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -613,16 +621,16 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2599/overview/1931f35c-87fe-4b6a-a718-a61a2d00e86a</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/bridgeai-deployment-catalyst-ai-for-operational-systems/</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-10-06 16:27</t>
+          <t>2026-10-10 15:37</t>
         </is>
       </c>
       <c r="E4" s="1" t="n">
-        <v>46301.68541666667</v>
+        <v>46305.65069444444</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
@@ -631,11 +639,17 @@
       <c r="H4" t="b">
         <v>0</v>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>21/10/2026</t>
+        </is>
+      </c>
+      <c r="J4" s="1" t="n">
+        <v>46316</v>
+      </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Tuesday 8 December 2026 11:00am</t>
+          <t>08/12/2026                              11:00</t>
         </is>
       </c>
       <c r="L4" s="1" t="n">
@@ -643,11 +657,11 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>£200,000</t>
+          <t>£52.0 million</t>
         </is>
       </c>
       <c r="N4" s="1" t="n">
-        <v>46295</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="5">
@@ -658,21 +672,21 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Eureka collaborative R&amp;D: Globalstars Japan 2027</t>
+          <t>BridgeAI Deployment Catalyst: AI for Decision Critical Systems</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/eureka-collaborative-rd-globalstars-japan-2027/</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/bridgeai-deployment-catalyst-ai-for-decision-critical-systems/</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-10-06 16:20</t>
+          <t>2026-10-10 15:37</t>
         </is>
       </c>
       <c r="E5" s="1" t="n">
-        <v>46301.68055555555</v>
+        <v>46305.65069444444</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
@@ -683,27 +697,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="J5" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>08/12/2026                              11:00</t>
+        </is>
+      </c>
+      <c r="L5" s="1" t="n">
+        <v>46364.45833333334</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>£52.0 million</t>
+        </is>
+      </c>
+      <c r="N5" s="1" t="n">
         <v>46302</v>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>20/01/2027                              11:00</t>
-        </is>
-      </c>
-      <c r="L5" s="1" t="n">
-        <v>46407.45833333334</v>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>£2.0 million</t>
-        </is>
-      </c>
-      <c r="N5" s="1" t="n">
-        <v>46295</v>
       </c>
     </row>
     <row r="6">
@@ -714,21 +728,21 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Next Wave: Global Business Innovation Programme – Createch South by Southwest (SXSW), Texas</t>
+          <t>BridgeAI Deployment Catalyst: AI for Assurance and Compliance</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/next-wave-gbip-createch-sxsw-texas/</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/bridgeai-deployment-catalyst-ai-for-assurance-and-compliance/</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-10-06 16:20</t>
+          <t>2026-10-10 15:37</t>
         </is>
       </c>
       <c r="E6" s="1" t="n">
-        <v>46301.68055555555</v>
+        <v>46305.65069444444</v>
       </c>
       <c r="F6" t="b">
         <v>1</v>
@@ -739,21 +753,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="J6" s="1" t="n">
-        <v>46301</v>
+        <v>46316</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
+          <t>08/12/2026                              11:00</t>
+        </is>
+      </c>
+      <c r="L6" s="1" t="n">
+        <v>46364.45833333334</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>£52.0 million</t>
+        </is>
+      </c>
       <c r="N6" s="1" t="n">
-        <v>46295</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="7">
@@ -764,21 +784,21 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ADOPT Facilitator Support Grant: Round 12</t>
+          <t>iX Challenge: Accelerating Digital Engineering Through MBSE Simulation</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/adopt-facilitator-support-grant-round-12/</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/ix-challenge-accelerating-digital-engineering-through-mbse-simulation/</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-06 16:20</t>
+          <t>2026-10-09 16:39</t>
         </is>
       </c>
       <c r="E7" s="1" t="n">
-        <v>46301.68055555555</v>
+        <v>46304.69375</v>
       </c>
       <c r="F7" t="b">
         <v>1</v>
@@ -789,27 +809,25 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="J7" s="1" t="n">
-        <v>46296</v>
+        <v>46304</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>11/11/2026                              11:00</t>
-        </is>
-      </c>
-      <c r="L7" s="1" t="n">
-        <v>46337.45833333334</v>
-      </c>
+          <t>06/11/2026</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
-          <t>£200,000</t>
+          <t>£60,000</t>
         </is>
       </c>
       <c r="N7" s="1" t="n">
-        <v>46295</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="8">
@@ -820,21 +838,21 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>iX Challenge: AI Attribution and AI Authenticity for Ethical Cultural Content</t>
+          <t>Full ADOPT Grant: Round 10</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/ix-challenge-ai-attribution-and-ai-authenticity-for-ethical-cultural-content/</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/full-adopt-grant-round-10/</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-10-06 16:20</t>
+          <t>2026-10-09 16:39</t>
         </is>
       </c>
       <c r="E8" s="1" t="n">
-        <v>46301.68055555555</v>
+        <v>46304.69375</v>
       </c>
       <c r="F8" t="b">
         <v>1</v>
@@ -845,25 +863,27 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="J8" s="1" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>13/11/2026</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr"/>
+          <t>02/12/2026                              11:00</t>
+        </is>
+      </c>
+      <c r="L8" s="1" t="n">
+        <v>46358.45833333334</v>
+      </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>£50,000</t>
+          <t>£5.0 million</t>
         </is>
       </c>
       <c r="N8" s="1" t="n">
-        <v>46295</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="9">
@@ -874,21 +894,21 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Investor Partnerships – Battery Innovation Programme</t>
+          <t>iX Challenge: Repeatable Adversarial Evaluation of Physical Tamper Protection for Defence Electronics</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/investor-partnerships-battery-innovation-programme/</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/ix-challenge-repeatable-adversarial-evaluation-of-physical-tamper-protection-for-defence-electronics/</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-06 16:20</t>
+          <t>2026-10-09 16:39</t>
         </is>
       </c>
       <c r="E9" s="1" t="n">
-        <v>46301.68055555555</v>
+        <v>46304.69375</v>
       </c>
       <c r="F9" t="b">
         <v>1</v>
@@ -899,52 +919,50 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>05/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="J9" s="1" t="n">
-        <v>46300</v>
+        <v>46304</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>25/11/2026                              11:00</t>
-        </is>
-      </c>
-      <c r="L9" s="1" t="n">
-        <v>46351.45833333334</v>
-      </c>
+          <t>06/11/2026</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr">
         <is>
-          <t>£2.0 million</t>
+          <t>£60,000</t>
         </is>
       </c>
       <c r="N9" s="1" t="n">
-        <v>46295</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Innovate UK Business Connect</t>
+          <t>Innovate Funding Service</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Sustainable Medicines Manufacturing Innovation: CR&amp;D Round 2</t>
+          <t>Full ADOPT Grant: Round 10</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/sustainable-medicines-manufacturing-innovation-crd-round-2/</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2596/overview/31f0a768-2a9a-405d-b0a4-83a8c5b395c0</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-06 16:20</t>
+          <t>2026-10-08 17:07</t>
         </is>
       </c>
       <c r="E10" s="1" t="n">
-        <v>46301.68055555555</v>
+        <v>46303.71319444444</v>
       </c>
       <c r="F10" t="b">
         <v>1</v>
@@ -953,17 +971,11 @@
       <c r="H10" t="b">
         <v>0</v>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>05/10/2026</t>
-        </is>
-      </c>
-      <c r="J10" s="1" t="n">
-        <v>46300</v>
-      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>02/12/2026                              11:00</t>
+          <t>Wednesday 2 December 2026 11:00am</t>
         </is>
       </c>
       <c r="L10" s="1" t="n">
@@ -971,36 +983,36 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>£7.0 million</t>
+          <t>£200,000</t>
         </is>
       </c>
       <c r="N10" s="1" t="n">
-        <v>46295</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Innovate Funding Service</t>
+          <t>Innovate UK Business Connect</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Eureka collaborative R&amp;D: Globalstars Japan 2027</t>
+          <t>iX Challenge: Reducing blood-cell loss and measurement variability in field-deployable microfluidic diagnostic cartridges</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2586/overview/d9e61ae4-6e56-4f38-9206-5d91ef98c916</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/ix-challenge-reducing-blood-cell-loss-and-measurement-variability-in-field-deployable-microfluidic-diagnostic-cartridges/</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-10-05 19:06</t>
+          <t>2026-10-08 17:01</t>
         </is>
       </c>
       <c r="E11" s="1" t="n">
-        <v>46300.79583333333</v>
+        <v>46303.70902777778</v>
       </c>
       <c r="F11" t="b">
         <v>1</v>
@@ -1009,48 +1021,54 @@
       <c r="H11" t="b">
         <v>0</v>
       </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="J11" s="1" t="n">
+        <v>46300</v>
+      </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Wednesday 20 January 2027 11:00am</t>
+          <t>06/11/2026                              11:00</t>
         </is>
       </c>
       <c r="L11" s="1" t="n">
-        <v>46407.45833333334</v>
+        <v>46332.45833333334</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>£600,000</t>
+          <t>£60,000</t>
         </is>
       </c>
       <c r="N11" s="1" t="n">
-        <v>46295</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Innovate Funding Service</t>
+          <t>Innovate UK Business Connect</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Sustainable Medicines Manufacturing Innovation: CR&amp;D Round 2</t>
+          <t>FOAK Builder: working towards climate tech first-of-a-kind deployment</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2560/overview/45acacd5-746b-46ee-8051-d764f929cca3</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/foak-builder-working-towards-climate-tech-first-of-a-kind-deployment/</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-10-05 19:06</t>
+          <t>2026-10-08 17:01</t>
         </is>
       </c>
       <c r="E12" s="1" t="n">
-        <v>46300.79583333333</v>
+        <v>46303.70902777778</v>
       </c>
       <c r="F12" t="b">
         <v>1</v>
@@ -1059,48 +1077,54 @@
       <c r="H12" t="b">
         <v>0</v>
       </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="J12" s="1" t="n">
+        <v>46302</v>
+      </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Wednesday 2 December 2026 11:00am</t>
+          <t>05/11/2026                              11:00</t>
         </is>
       </c>
       <c r="L12" s="1" t="n">
-        <v>46358.45833333334</v>
+        <v>46331.45833333334</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>£1.0 million</t>
+          <t>£4.8 million</t>
         </is>
       </c>
       <c r="N12" s="1" t="n">
-        <v>46295</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Innovate Funding Service</t>
+          <t>Innovate UK Business Connect</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Investor Partnerships – Battery Innovation Programme</t>
+          <t>iX Challenge: Verified reporting of the value created by defence contracts</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2595/overview/f2b849f6-0fb3-4012-be1b-a41813c93085</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/ix-challenge-verified-reporting-of-the-value-created-by-defence-contracts/</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-10-05 19:06</t>
+          <t>2026-10-08 17:01</t>
         </is>
       </c>
       <c r="E13" s="1" t="n">
-        <v>46300.79583333333</v>
+        <v>46303.70902777778</v>
       </c>
       <c r="F13" t="b">
         <v>1</v>
@@ -1109,48 +1133,52 @@
       <c r="H13" t="b">
         <v>0</v>
       </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="J13" s="1" t="n">
+        <v>46300</v>
+      </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Wednesday 25 November 2026 11:00am</t>
-        </is>
-      </c>
-      <c r="L13" s="1" t="n">
-        <v>46351.45833333334</v>
-      </c>
+          <t>06/11/2026</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr">
         <is>
-          <t>£2.0 million</t>
+          <t>£60,000</t>
         </is>
       </c>
       <c r="N13" s="1" t="n">
-        <v>46295</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Innovate Funding Service</t>
+          <t>Innovate UK Business Connect</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ADOPT Facilitator Support Grant: Round 12</t>
+          <t>iX Challenge: Extending protection to personnel travelling in armoured vehicles under drone attack</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2591/overview/b66dd413-9894-4fc4-a6c9-cced53367568</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/ix-challenge-extending-protection-to-personnel-travelling-in-armoured-vehicles-under-drone-attack/</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-10-05 19:06</t>
+          <t>2026-10-08 17:01</t>
         </is>
       </c>
       <c r="E14" s="1" t="n">
-        <v>46300.79583333333</v>
+        <v>46303.70902777778</v>
       </c>
       <c r="F14" t="b">
         <v>1</v>
@@ -1159,23 +1187,27 @@
       <c r="H14" t="b">
         <v>0</v>
       </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="J14" s="1" t="n">
+        <v>46300</v>
+      </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Wednesday 11 November 2026 11:00am</t>
-        </is>
-      </c>
-      <c r="L14" s="1" t="n">
-        <v>46337.45833333334</v>
-      </c>
+          <t>06/11/2026</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr">
         <is>
-          <t>£2,500</t>
+          <t>£60,000</t>
         </is>
       </c>
       <c r="N14" s="1" t="n">
-        <v>46295</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="15">
@@ -1186,21 +1218,21 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>HMGCC Co-Creation Challenge: Hidden stab vests for women</t>
+          <t>iX Challenge: Edge AI with Low Size, Weight, Power, and Cost</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/hmgcc-co-creation-challenge-hidden-stab-vests-for-women/</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/ix-challenge-edge-ai-with-low-size-weight-power-and-cost/</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-10-05 18:54</t>
+          <t>2026-10-08 17:01</t>
         </is>
       </c>
       <c r="E15" s="1" t="n">
-        <v>46300.7875</v>
+        <v>46303.70902777778</v>
       </c>
       <c r="F15" t="b">
         <v>1</v>
@@ -1219,19 +1251,17 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>05/11/2026                              12:00</t>
-        </is>
-      </c>
-      <c r="L15" s="1" t="n">
-        <v>46331.5</v>
-      </c>
+          <t>06/11/2026</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr">
         <is>
           <t>£60,000</t>
         </is>
       </c>
       <c r="N15" s="1" t="n">
-        <v>46295</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="16">
@@ -1242,21 +1272,21 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Engineering Biology Investor Partnerships Round 1</t>
+          <t>iX Challenge: Resilient High-Altitude Communications, Navigation and Mission Connectivity for Persistent Autonomous Aircraft</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/engineering-biology-investor-partnerships-round-1/</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/ix-challenge-resilient-high-altitude-communications-navigation-and-mission-connectivity-for-persistent-autonomous-aircraft/</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-10-05 18:54</t>
+          <t>2026-10-08 17:01</t>
         </is>
       </c>
       <c r="E16" s="1" t="n">
-        <v>46300.7875</v>
+        <v>46303.70902777778</v>
       </c>
       <c r="F16" t="b">
         <v>1</v>
@@ -1267,27 +1297,25 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>05/10/2026</t>
         </is>
       </c>
       <c r="J16" s="1" t="n">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>02/12/2026                              11:00</t>
-        </is>
-      </c>
-      <c r="L16" s="1" t="n">
-        <v>46358.45833333334</v>
-      </c>
+          <t>06/11/2026</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr">
         <is>
-          <t>£8.0 million</t>
+          <t>£60,000</t>
         </is>
       </c>
       <c r="N16" s="1" t="n">
-        <v>46295</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="17">
@@ -1298,21 +1326,21 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Manufacturing Digitalisation Innovation Programme: Innovation and Scale-up Hub</t>
+          <t>iX Challenge: Distributed Smartphone-Based Detection and Mapping of PNT Signal Interference</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/mdi-programme-innovation-and-scale-up-hub/</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/ix-challenge-distributed-smartphone-based-detection-and-mapping-of-pnt-signal-interference/</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-10-05 18:54</t>
+          <t>2026-10-08 17:01</t>
         </is>
       </c>
       <c r="E17" s="1" t="n">
-        <v>46300.7875</v>
+        <v>46303.70902777778</v>
       </c>
       <c r="F17" t="b">
         <v>1</v>
@@ -1323,52 +1351,50 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>02/10/2026</t>
+          <t>05/10/2026</t>
         </is>
       </c>
       <c r="J17" s="1" t="n">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>18/11/2026                              11:00</t>
-        </is>
-      </c>
-      <c r="L17" s="1" t="n">
-        <v>46344.45833333334</v>
-      </c>
+          <t>06/11/2026</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr">
         <is>
-          <t>£175.0 million</t>
+          <t>£60,000</t>
         </is>
       </c>
       <c r="N17" s="1" t="n">
-        <v>46295</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Innovate Funding Service</t>
+          <t>Innovate UK Business Connect</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>MDI Programme Innovation and Scale-up Hub</t>
+          <t>iX Challenge: Secure, Cost-Effective Use of Cloud-Based AI Tools in the Defence Supply Chain</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2588/overview/acbd9666-c1df-4635-b86f-fa426100c876</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/ix-challenge-secure-cost-effective-use-of-cloud-based-ai-tools-in-the-defence-supply-chain/</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-10-03 14:31</t>
+          <t>2026-10-08 17:01</t>
         </is>
       </c>
       <c r="E18" s="1" t="n">
-        <v>46298.60486111111</v>
+        <v>46303.70902777778</v>
       </c>
       <c r="F18" t="b">
         <v>1</v>
@@ -1377,48 +1403,52 @@
       <c r="H18" t="b">
         <v>0</v>
       </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="J18" s="1" t="n">
+        <v>46300</v>
+      </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Wednesday 18 November 2026 11:00am</t>
-        </is>
-      </c>
-      <c r="L18" s="1" t="n">
-        <v>46344.45833333334</v>
-      </c>
+          <t>06/11/2026</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr">
         <is>
-          <t>£4.0 million</t>
+          <t>£60,000</t>
         </is>
       </c>
       <c r="N18" s="1" t="n">
-        <v>46295</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Innovate Funding Service</t>
+          <t>Innovate UK Business Connect</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Engineering Biology Investor Partnerships Round 1</t>
+          <t>iX Challenge: Next-Generation Electronics for UK Bathymetric Sonar</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2580/overview/8881af18-31f4-4db3-9483-cbb047163164</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/ix-challenge-next-generation-electronics-for-uk-bathymetric-sonar/</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-10-01 16:50</t>
+          <t>2026-10-08 17:01</t>
         </is>
       </c>
       <c r="E19" s="1" t="n">
-        <v>46296.70138888889</v>
+        <v>46303.70902777778</v>
       </c>
       <c r="F19" t="b">
         <v>1</v>
@@ -1427,48 +1457,52 @@
       <c r="H19" t="b">
         <v>0</v>
       </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="J19" s="1" t="n">
+        <v>46302</v>
+      </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Wednesday 2 December 2026 11:00am</t>
-        </is>
-      </c>
-      <c r="L19" s="1" t="n">
-        <v>46358.45833333334</v>
-      </c>
+          <t>06/11/2026</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr">
         <is>
-          <t>£2.0 million</t>
+          <t>£60,000</t>
         </is>
       </c>
       <c r="N19" s="1" t="n">
-        <v>46295</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Innovate UK Business Connect</t>
+          <t>Innovate Funding Service</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>UKAEA ICURe Engage - November 2026</t>
+          <t>FOAK Builder: Programme Entry Expression of Interest</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/ukaea-icure-engage-november-2026/</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2600/overview/0c422454-a8af-4c24-a74a-565426f42395</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-10-01 16:44</t>
+          <t>2026-10-07 17:10</t>
         </is>
       </c>
       <c r="E20" s="1" t="n">
-        <v>46296.69722222222</v>
+        <v>46302.71527777778</v>
       </c>
       <c r="F20" t="b">
         <v>1</v>
@@ -1477,81 +1511,23 @@
       <c r="H20" t="b">
         <v>0</v>
       </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>02/10/2026</t>
-        </is>
-      </c>
-      <c r="J20" s="1" t="n">
-        <v>46297</v>
-      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
-          <t>29/10/2026                              11:59</t>
+          <t>Thursday 5 November 2026 11:00am</t>
         </is>
       </c>
       <c r="L20" s="1" t="n">
-        <v>46324.49930555555</v>
-      </c>
-      <c r="M20" t="inlineStr"/>
+        <v>46331.45833333334</v>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>£100.0 million</t>
+        </is>
+      </c>
       <c r="N20" s="1" t="n">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Innovate UK Business Connect</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>UK Defence Innovation: Security Open Call 2026 Cycle 2</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/uk-defence-innovation-security-open-call-2026-cycle-2/</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>2026-10-01 16:44</t>
-        </is>
-      </c>
-      <c r="E21" s="1" t="n">
-        <v>46296.69722222222</v>
-      </c>
-      <c r="F21" t="b">
-        <v>1</v>
-      </c>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="b">
-        <v>0</v>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-      <c r="J21" s="1" t="n">
-        <v>46296</v>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>29/10/2026                              12:00</t>
-        </is>
-      </c>
-      <c r="L21" s="1" t="n">
-        <v>46324.5</v>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>£350,000</t>
-        </is>
-      </c>
-      <c r="N21" s="1" t="n">
-        <v>46295</v>
+        <v>46302</v>
       </c>
     </row>
   </sheetData>
@@ -1565,7 +1541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1643,26 +1619,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Innovate UK Business Connect</t>
+          <t>Innovate Funding Service</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>HMGCC Co-Creation Challenge: Multi-Terrain Micro Robotic Systems</t>
+          <t>Growth Cohorts: Next-gen low carbon concrete cohort entry Round 2</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/hmgcc-co-creation-challenge-multi-terrain-micro-robotic-systems/</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2602/overview/607351e2-798f-450b-b77d-3131912bcbef</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-12 19:27</t>
+          <t>2026-10-14 14:50</t>
         </is>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46307.81041666667</v>
+        <v>46309.61805555555</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
@@ -1671,1003 +1647,23 @@
       <c r="H2" t="b">
         <v>0</v>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>12/10/2026</t>
-        </is>
-      </c>
-      <c r="J2" s="1" t="n">
-        <v>46307</v>
-      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>12/11/2026</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
+          <t>Wednesday 2 December 2026 11:00am</t>
+        </is>
+      </c>
+      <c r="L2" s="1" t="n">
+        <v>46358.45833333334</v>
+      </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>£60,000</t>
+          <t>£54,400</t>
         </is>
       </c>
       <c r="N2" s="1" t="n">
-        <v>46302</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Innovate UK Business Connect</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>HMGCC Co-Creation Challenge: Smart glasses for mapping</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/hmgcc-co-creation-challenge-smart-glasses-for-mapping/</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2026-10-12 19:27</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="n">
-        <v>46307.81041666667</v>
-      </c>
-      <c r="F3" t="b">
-        <v>1</v>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="b">
-        <v>0</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>12/10/2026</t>
-        </is>
-      </c>
-      <c r="J3" s="1" t="n">
-        <v>46307</v>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>12/11/2026</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>£60,000</t>
-        </is>
-      </c>
-      <c r="N3" s="1" t="n">
-        <v>46302</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Innovate UK Business Connect</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>BridgeAI Deployment Catalyst: AI for Operational Systems</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/bridgeai-deployment-catalyst-ai-for-operational-systems/</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2026-10-10 15:37</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="n">
-        <v>46305.65069444444</v>
-      </c>
-      <c r="F4" t="b">
-        <v>1</v>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="b">
-        <v>0</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>21/10/2026</t>
-        </is>
-      </c>
-      <c r="J4" s="1" t="n">
-        <v>46316</v>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>08/12/2026                              11:00</t>
-        </is>
-      </c>
-      <c r="L4" s="1" t="n">
-        <v>46364.45833333334</v>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>£52.0 million</t>
-        </is>
-      </c>
-      <c r="N4" s="1" t="n">
-        <v>46302</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Innovate UK Business Connect</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>BridgeAI Deployment Catalyst: AI for Decision Critical Systems</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/bridgeai-deployment-catalyst-ai-for-decision-critical-systems/</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>2026-10-10 15:37</t>
-        </is>
-      </c>
-      <c r="E5" s="1" t="n">
-        <v>46305.65069444444</v>
-      </c>
-      <c r="F5" t="b">
-        <v>1</v>
-      </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="b">
-        <v>0</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>21/10/2026</t>
-        </is>
-      </c>
-      <c r="J5" s="1" t="n">
-        <v>46316</v>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>08/12/2026                              11:00</t>
-        </is>
-      </c>
-      <c r="L5" s="1" t="n">
-        <v>46364.45833333334</v>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>£52.0 million</t>
-        </is>
-      </c>
-      <c r="N5" s="1" t="n">
-        <v>46302</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Innovate UK Business Connect</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>BridgeAI Deployment Catalyst: AI for Assurance and Compliance</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/bridgeai-deployment-catalyst-ai-for-assurance-and-compliance/</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>2026-10-10 15:37</t>
-        </is>
-      </c>
-      <c r="E6" s="1" t="n">
-        <v>46305.65069444444</v>
-      </c>
-      <c r="F6" t="b">
-        <v>1</v>
-      </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="b">
-        <v>0</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>21/10/2026</t>
-        </is>
-      </c>
-      <c r="J6" s="1" t="n">
-        <v>46316</v>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>08/12/2026                              11:00</t>
-        </is>
-      </c>
-      <c r="L6" s="1" t="n">
-        <v>46364.45833333334</v>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>£52.0 million</t>
-        </is>
-      </c>
-      <c r="N6" s="1" t="n">
-        <v>46302</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Innovate UK Business Connect</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>iX Challenge: Accelerating Digital Engineering Through MBSE Simulation</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/ix-challenge-accelerating-digital-engineering-through-mbse-simulation/</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>2026-10-09 16:39</t>
-        </is>
-      </c>
-      <c r="E7" s="1" t="n">
-        <v>46304.69375</v>
-      </c>
-      <c r="F7" t="b">
-        <v>1</v>
-      </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="b">
-        <v>0</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>09/10/2026</t>
-        </is>
-      </c>
-      <c r="J7" s="1" t="n">
-        <v>46304</v>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>06/11/2026</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>£60,000</t>
-        </is>
-      </c>
-      <c r="N7" s="1" t="n">
-        <v>46302</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Innovate UK Business Connect</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Full ADOPT Grant: Round 10</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/full-adopt-grant-round-10/</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>2026-10-09 16:39</t>
-        </is>
-      </c>
-      <c r="E8" s="1" t="n">
-        <v>46304.69375</v>
-      </c>
-      <c r="F8" t="b">
-        <v>1</v>
-      </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="b">
-        <v>0</v>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>08/10/2026</t>
-        </is>
-      </c>
-      <c r="J8" s="1" t="n">
-        <v>46303</v>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>02/12/2026                              11:00</t>
-        </is>
-      </c>
-      <c r="L8" s="1" t="n">
-        <v>46358.45833333334</v>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>£5.0 million</t>
-        </is>
-      </c>
-      <c r="N8" s="1" t="n">
-        <v>46302</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Innovate UK Business Connect</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>iX Challenge: Repeatable Adversarial Evaluation of Physical Tamper Protection for Defence Electronics</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/ix-challenge-repeatable-adversarial-evaluation-of-physical-tamper-protection-for-defence-electronics/</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>2026-10-09 16:39</t>
-        </is>
-      </c>
-      <c r="E9" s="1" t="n">
-        <v>46304.69375</v>
-      </c>
-      <c r="F9" t="b">
-        <v>1</v>
-      </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="b">
-        <v>0</v>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>09/10/2026</t>
-        </is>
-      </c>
-      <c r="J9" s="1" t="n">
-        <v>46304</v>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>06/11/2026</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>£60,000</t>
-        </is>
-      </c>
-      <c r="N9" s="1" t="n">
-        <v>46302</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Innovate Funding Service</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Full ADOPT Grant: Round 10</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2596/overview/31f0a768-2a9a-405d-b0a4-83a8c5b395c0</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>2026-10-08 17:07</t>
-        </is>
-      </c>
-      <c r="E10" s="1" t="n">
-        <v>46303.71319444444</v>
-      </c>
-      <c r="F10" t="b">
-        <v>1</v>
-      </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="b">
-        <v>0</v>
-      </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>Wednesday 2 December 2026 11:00am</t>
-        </is>
-      </c>
-      <c r="L10" s="1" t="n">
-        <v>46358.45833333334</v>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>£200,000</t>
-        </is>
-      </c>
-      <c r="N10" s="1" t="n">
-        <v>46302</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Innovate UK Business Connect</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>iX Challenge: Reducing blood-cell loss and measurement variability in field-deployable microfluidic diagnostic cartridges</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/ix-challenge-reducing-blood-cell-loss-and-measurement-variability-in-field-deployable-microfluidic-diagnostic-cartridges/</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>2026-10-08 17:01</t>
-        </is>
-      </c>
-      <c r="E11" s="1" t="n">
-        <v>46303.70902777778</v>
-      </c>
-      <c r="F11" t="b">
-        <v>1</v>
-      </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="b">
-        <v>0</v>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>05/10/2026</t>
-        </is>
-      </c>
-      <c r="J11" s="1" t="n">
-        <v>46300</v>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>06/11/2026                              11:00</t>
-        </is>
-      </c>
-      <c r="L11" s="1" t="n">
-        <v>46332.45833333334</v>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>£60,000</t>
-        </is>
-      </c>
-      <c r="N11" s="1" t="n">
-        <v>46302</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Innovate UK Business Connect</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>FOAK Builder: working towards climate tech first-of-a-kind deployment</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/foak-builder-working-towards-climate-tech-first-of-a-kind-deployment/</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>2026-10-08 17:01</t>
-        </is>
-      </c>
-      <c r="E12" s="1" t="n">
-        <v>46303.70902777778</v>
-      </c>
-      <c r="F12" t="b">
-        <v>1</v>
-      </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="b">
-        <v>0</v>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>07/10/2026</t>
-        </is>
-      </c>
-      <c r="J12" s="1" t="n">
-        <v>46302</v>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>05/11/2026                              11:00</t>
-        </is>
-      </c>
-      <c r="L12" s="1" t="n">
-        <v>46331.45833333334</v>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>£4.8 million</t>
-        </is>
-      </c>
-      <c r="N12" s="1" t="n">
-        <v>46302</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Innovate UK Business Connect</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>iX Challenge: Verified reporting of the value created by defence contracts</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/ix-challenge-verified-reporting-of-the-value-created-by-defence-contracts/</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>2026-10-08 17:01</t>
-        </is>
-      </c>
-      <c r="E13" s="1" t="n">
-        <v>46303.70902777778</v>
-      </c>
-      <c r="F13" t="b">
-        <v>1</v>
-      </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="b">
-        <v>0</v>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>05/10/2026</t>
-        </is>
-      </c>
-      <c r="J13" s="1" t="n">
-        <v>46300</v>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>06/11/2026</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>£60,000</t>
-        </is>
-      </c>
-      <c r="N13" s="1" t="n">
-        <v>46302</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Innovate UK Business Connect</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>iX Challenge: Extending protection to personnel travelling in armoured vehicles under drone attack</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/ix-challenge-extending-protection-to-personnel-travelling-in-armoured-vehicles-under-drone-attack/</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>2026-10-08 17:01</t>
-        </is>
-      </c>
-      <c r="E14" s="1" t="n">
-        <v>46303.70902777778</v>
-      </c>
-      <c r="F14" t="b">
-        <v>1</v>
-      </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="b">
-        <v>0</v>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>05/10/2026</t>
-        </is>
-      </c>
-      <c r="J14" s="1" t="n">
-        <v>46300</v>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>06/11/2026</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>£60,000</t>
-        </is>
-      </c>
-      <c r="N14" s="1" t="n">
-        <v>46302</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Innovate UK Business Connect</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>iX Challenge: Edge AI with Low Size, Weight, Power, and Cost</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/ix-challenge-edge-ai-with-low-size-weight-power-and-cost/</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>2026-10-08 17:01</t>
-        </is>
-      </c>
-      <c r="E15" s="1" t="n">
-        <v>46303.70902777778</v>
-      </c>
-      <c r="F15" t="b">
-        <v>1</v>
-      </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="b">
-        <v>0</v>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>05/10/2026</t>
-        </is>
-      </c>
-      <c r="J15" s="1" t="n">
-        <v>46300</v>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>06/11/2026</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>£60,000</t>
-        </is>
-      </c>
-      <c r="N15" s="1" t="n">
-        <v>46302</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Innovate UK Business Connect</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>iX Challenge: Resilient High-Altitude Communications, Navigation and Mission Connectivity for Persistent Autonomous Aircraft</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/ix-challenge-resilient-high-altitude-communications-navigation-and-mission-connectivity-for-persistent-autonomous-aircraft/</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>2026-10-08 17:01</t>
-        </is>
-      </c>
-      <c r="E16" s="1" t="n">
-        <v>46303.70902777778</v>
-      </c>
-      <c r="F16" t="b">
-        <v>1</v>
-      </c>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="b">
-        <v>0</v>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>05/10/2026</t>
-        </is>
-      </c>
-      <c r="J16" s="1" t="n">
-        <v>46300</v>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>06/11/2026</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>£60,000</t>
-        </is>
-      </c>
-      <c r="N16" s="1" t="n">
-        <v>46302</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Innovate UK Business Connect</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>iX Challenge: Distributed Smartphone-Based Detection and Mapping of PNT Signal Interference</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/ix-challenge-distributed-smartphone-based-detection-and-mapping-of-pnt-signal-interference/</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>2026-10-08 17:01</t>
-        </is>
-      </c>
-      <c r="E17" s="1" t="n">
-        <v>46303.70902777778</v>
-      </c>
-      <c r="F17" t="b">
-        <v>1</v>
-      </c>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="b">
-        <v>0</v>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>05/10/2026</t>
-        </is>
-      </c>
-      <c r="J17" s="1" t="n">
-        <v>46300</v>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>06/11/2026</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>£60,000</t>
-        </is>
-      </c>
-      <c r="N17" s="1" t="n">
-        <v>46302</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Innovate UK Business Connect</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>iX Challenge: Secure, Cost-Effective Use of Cloud-Based AI Tools in the Defence Supply Chain</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/ix-challenge-secure-cost-effective-use-of-cloud-based-ai-tools-in-the-defence-supply-chain/</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>2026-10-08 17:01</t>
-        </is>
-      </c>
-      <c r="E18" s="1" t="n">
-        <v>46303.70902777778</v>
-      </c>
-      <c r="F18" t="b">
-        <v>1</v>
-      </c>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="b">
-        <v>0</v>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>05/10/2026</t>
-        </is>
-      </c>
-      <c r="J18" s="1" t="n">
-        <v>46300</v>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>06/11/2026</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>£60,000</t>
-        </is>
-      </c>
-      <c r="N18" s="1" t="n">
-        <v>46302</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Innovate UK Business Connect</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>iX Challenge: Next-Generation Electronics for UK Bathymetric Sonar</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/ix-challenge-next-generation-electronics-for-uk-bathymetric-sonar/</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>2026-10-08 17:01</t>
-        </is>
-      </c>
-      <c r="E19" s="1" t="n">
-        <v>46303.70902777778</v>
-      </c>
-      <c r="F19" t="b">
-        <v>1</v>
-      </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="b">
-        <v>0</v>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>07/10/2026</t>
-        </is>
-      </c>
-      <c r="J19" s="1" t="n">
-        <v>46302</v>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>06/11/2026</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>£60,000</t>
-        </is>
-      </c>
-      <c r="N19" s="1" t="n">
-        <v>46302</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Innovate Funding Service</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>FOAK Builder: Programme Entry Expression of Interest</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2600/overview/0c422454-a8af-4c24-a74a-565426f42395</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>2026-10-07 17:10</t>
-        </is>
-      </c>
-      <c r="E20" s="1" t="n">
-        <v>46302.71527777778</v>
-      </c>
-      <c r="F20" t="b">
-        <v>1</v>
-      </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="b">
-        <v>0</v>
-      </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>Thursday 5 November 2026 11:00am</t>
-        </is>
-      </c>
-      <c r="L20" s="1" t="n">
-        <v>46331.45833333334</v>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>£100.0 million</t>
-        </is>
-      </c>
-      <c r="N20" s="1" t="n">
-        <v>46302</v>
+        <v>46309</v>
       </c>
     </row>
   </sheetData>
@@ -2681,7 +1677,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D71"/>
+  <dimension ref="A1:D72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2708,83 +1704,83 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46302</v>
+        <v>46309</v>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46295</v>
+        <v>46302</v>
       </c>
       <c r="B3" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="D3" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46288</v>
+        <v>46295</v>
       </c>
       <c r="B4" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C4" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46281</v>
+        <v>46288</v>
       </c>
       <c r="B5" t="n">
-        <v>32</v>
+        <v>5</v>
       </c>
       <c r="C5" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D5" t="n">
-        <v>48</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46274</v>
+        <v>46281</v>
       </c>
       <c r="B6" t="n">
-        <v>4</v>
+        <v>32</v>
       </c>
       <c r="C6" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D6" t="n">
-        <v>14</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46267</v>
+        <v>46274</v>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C7" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D7" t="n">
         <v>14</v>
@@ -2792,189 +1788,189 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46260</v>
+        <v>46267</v>
       </c>
       <c r="B8" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C8" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="D8" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46253</v>
+        <v>46260</v>
       </c>
       <c r="B9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D9" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46246</v>
+        <v>46253</v>
       </c>
       <c r="B10" t="n">
         <v>3</v>
       </c>
       <c r="C10" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D10" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46239</v>
+        <v>46246</v>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C11" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="D11" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46232</v>
+        <v>46239</v>
       </c>
       <c r="B12" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C12" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="D12" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46225</v>
+        <v>46232</v>
       </c>
       <c r="B13" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C13" t="n">
-        <v>118</v>
+        <v>2</v>
       </c>
       <c r="D13" t="n">
-        <v>118</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46218</v>
+        <v>46225</v>
       </c>
       <c r="B14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>118</v>
       </c>
       <c r="D14" t="n">
-        <v>2</v>
+        <v>118</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46211</v>
+        <v>46218</v>
       </c>
       <c r="B15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C15" t="n">
         <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46204</v>
+        <v>46211</v>
       </c>
       <c r="B16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C16" t="n">
         <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46197</v>
+        <v>46204</v>
       </c>
       <c r="B17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C17" t="n">
         <v>0</v>
       </c>
       <c r="D17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46190</v>
+        <v>46197</v>
       </c>
       <c r="B18" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C18" t="n">
         <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46183</v>
+        <v>46190</v>
       </c>
       <c r="B19" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C19" t="n">
         <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46176</v>
+        <v>46183</v>
       </c>
       <c r="B20" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C20" t="n">
         <v>0</v>
       </c>
       <c r="D20" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46169</v>
+        <v>46176</v>
       </c>
       <c r="B21" t="n">
         <v>5</v>
@@ -2988,385 +1984,385 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46162</v>
+        <v>46169</v>
       </c>
       <c r="B22" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C22" t="n">
         <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46155</v>
+        <v>46162</v>
       </c>
       <c r="B23" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C23" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D23" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46148</v>
+        <v>46155</v>
       </c>
       <c r="B24" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" t="n">
         <v>4</v>
       </c>
-      <c r="C24" t="n">
-        <v>9</v>
-      </c>
       <c r="D24" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46141</v>
+        <v>46148</v>
       </c>
       <c r="B25" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C25" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D25" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46134</v>
+        <v>46141</v>
       </c>
       <c r="B26" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C26" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D26" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46127</v>
+        <v>46134</v>
       </c>
       <c r="B27" t="n">
         <v>4</v>
       </c>
       <c r="C27" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D27" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46120</v>
+        <v>46127</v>
       </c>
       <c r="B28" t="n">
         <v>4</v>
       </c>
       <c r="C28" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D28" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46113</v>
+        <v>46120</v>
       </c>
       <c r="B29" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C29" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D29" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46106</v>
+        <v>46113</v>
       </c>
       <c r="B30" t="n">
         <v>5</v>
       </c>
       <c r="C30" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D30" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46099</v>
+        <v>46106</v>
       </c>
       <c r="B31" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C31" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D31" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46092</v>
+        <v>46099</v>
       </c>
       <c r="B32" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C32" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D32" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46085</v>
+        <v>46092</v>
       </c>
       <c r="B33" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C33" t="n">
         <v>7</v>
       </c>
       <c r="D33" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46078</v>
+        <v>46085</v>
       </c>
       <c r="B34" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C34" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D34" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46071</v>
+        <v>46078</v>
       </c>
       <c r="B35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C35" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="D35" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46064</v>
+        <v>46071</v>
       </c>
       <c r="B36" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C36" t="n">
+        <v>6</v>
+      </c>
+      <c r="D36" t="n">
         <v>9</v>
-      </c>
-      <c r="D36" t="n">
-        <v>14</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46057</v>
+        <v>46064</v>
       </c>
       <c r="B37" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C37" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D37" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46050</v>
+        <v>46057</v>
       </c>
       <c r="B38" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C38" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D38" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46043</v>
+        <v>46050</v>
       </c>
       <c r="B39" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C39" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D39" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46036</v>
+        <v>46043</v>
       </c>
       <c r="B40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C40" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D40" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46029</v>
+        <v>46036</v>
       </c>
       <c r="B41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C41" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D41" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46022</v>
+        <v>46029</v>
       </c>
       <c r="B42" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C42" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="D42" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46015</v>
+        <v>46022</v>
       </c>
       <c r="B43" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C43" t="n">
         <v>1</v>
       </c>
       <c r="D43" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46008</v>
+        <v>46015</v>
       </c>
       <c r="B44" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C44" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D44" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46001</v>
+        <v>46008</v>
       </c>
       <c r="B45" t="n">
         <v>2</v>
       </c>
       <c r="C45" t="n">
-        <v>77</v>
+        <v>5</v>
       </c>
       <c r="D45" t="n">
-        <v>79</v>
+        <v>7</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>45994</v>
+        <v>46001</v>
       </c>
       <c r="B46" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C46" t="n">
-        <v>0</v>
+        <v>77</v>
       </c>
       <c r="D46" t="n">
-        <v>0</v>
+        <v>79</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>45987</v>
+        <v>45994</v>
       </c>
       <c r="B47" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C47" t="n">
         <v>0</v>
       </c>
       <c r="D47" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>45980</v>
+        <v>45987</v>
       </c>
       <c r="B48" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C48" t="n">
         <v>0</v>
       </c>
       <c r="D48" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>45973</v>
+        <v>45980</v>
       </c>
       <c r="B49" t="n">
         <v>0</v>
@@ -3380,91 +2376,91 @@
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>45966</v>
+        <v>45973</v>
       </c>
       <c r="B50" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C50" t="n">
         <v>0</v>
       </c>
       <c r="D50" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>45959</v>
+        <v>45966</v>
       </c>
       <c r="B51" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C51" t="n">
         <v>0</v>
       </c>
       <c r="D51" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>45952</v>
+        <v>45959</v>
       </c>
       <c r="B52" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C52" t="n">
         <v>0</v>
       </c>
       <c r="D52" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>45945</v>
+        <v>45952</v>
       </c>
       <c r="B53" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C53" t="n">
         <v>0</v>
       </c>
       <c r="D53" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>45938</v>
+        <v>45945</v>
       </c>
       <c r="B54" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C54" t="n">
         <v>0</v>
       </c>
       <c r="D54" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>45931</v>
+        <v>45938</v>
       </c>
       <c r="B55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C55" t="n">
         <v>0</v>
       </c>
       <c r="D55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>45924</v>
+        <v>45931</v>
       </c>
       <c r="B56" t="n">
         <v>1</v>
@@ -3478,35 +2474,35 @@
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>45917</v>
+        <v>45924</v>
       </c>
       <c r="B57" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C57" t="n">
         <v>0</v>
       </c>
       <c r="D57" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>45910</v>
+        <v>45917</v>
       </c>
       <c r="B58" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C58" t="n">
         <v>0</v>
       </c>
       <c r="D58" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>45903</v>
+        <v>45910</v>
       </c>
       <c r="B59" t="n">
         <v>2</v>
@@ -3520,169 +2516,183 @@
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>45896</v>
+        <v>45903</v>
       </c>
       <c r="B60" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C60" t="n">
         <v>0</v>
       </c>
       <c r="D60" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>45889</v>
+        <v>45896</v>
       </c>
       <c r="B61" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C61" t="n">
         <v>0</v>
       </c>
       <c r="D61" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>45882</v>
+        <v>45889</v>
       </c>
       <c r="B62" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C62" t="n">
         <v>0</v>
       </c>
       <c r="D62" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>45875</v>
+        <v>45882</v>
       </c>
       <c r="B63" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C63" t="n">
         <v>0</v>
       </c>
       <c r="D63" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>45868</v>
+        <v>45875</v>
       </c>
       <c r="B64" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C64" t="n">
         <v>0</v>
       </c>
       <c r="D64" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>45861</v>
+        <v>45868</v>
       </c>
       <c r="B65" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C65" t="n">
         <v>0</v>
       </c>
       <c r="D65" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>45854</v>
+        <v>45861</v>
       </c>
       <c r="B66" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C66" t="n">
         <v>0</v>
       </c>
       <c r="D66" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>45847</v>
+        <v>45854</v>
       </c>
       <c r="B67" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C67" t="n">
         <v>0</v>
       </c>
       <c r="D67" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>45840</v>
+        <v>45847</v>
       </c>
       <c r="B68" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C68" t="n">
         <v>0</v>
       </c>
       <c r="D68" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>45833</v>
+        <v>45840</v>
       </c>
       <c r="B69" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C69" t="n">
         <v>0</v>
       </c>
       <c r="D69" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>45826</v>
+        <v>45833</v>
       </c>
       <c r="B70" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C70" t="n">
         <v>0</v>
       </c>
       <c r="D70" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
+        <v>45826</v>
+      </c>
+      <c r="B71" t="n">
+        <v>0</v>
+      </c>
+      <c r="C71" t="n">
+        <v>0</v>
+      </c>
+      <c r="D71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
         <v>45819</v>
       </c>
-      <c r="B71" t="n">
+      <c r="B72" t="n">
         <v>25</v>
       </c>
-      <c r="C71" t="n">
-        <v>0</v>
-      </c>
-      <c r="D71" t="n">
+      <c r="C72" t="n">
+        <v>0</v>
+      </c>
+      <c r="D72" t="n">
         <v>25</v>
       </c>
     </row>
@@ -3697,7 +2707,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N730"/>
+  <dimension ref="A1:N731"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -40868,6 +39878,56 @@
       </c>
       <c r="N730" s="1" t="n">
         <v>46302</v>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>Innovate Funding Service</t>
+        </is>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>Growth Cohorts: Next-gen low carbon concrete cohort entry Round 2</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2602/overview/607351e2-798f-450b-b77d-3131912bcbef</t>
+        </is>
+      </c>
+      <c r="D731" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:50</t>
+        </is>
+      </c>
+      <c r="E731" s="1" t="n">
+        <v>46309.61805555555</v>
+      </c>
+      <c r="F731" t="b">
+        <v>1</v>
+      </c>
+      <c r="G731" t="inlineStr"/>
+      <c r="H731" t="b">
+        <v>0</v>
+      </c>
+      <c r="I731" t="inlineStr"/>
+      <c r="J731" t="inlineStr"/>
+      <c r="K731" t="inlineStr">
+        <is>
+          <t>Wednesday 2 December 2026 11:00am</t>
+        </is>
+      </c>
+      <c r="L731" s="1" t="n">
+        <v>46358.45833333334</v>
+      </c>
+      <c r="M731" t="inlineStr">
+        <is>
+          <t>£54,400</t>
+        </is>
+      </c>
+      <c r="N731" s="1" t="n">
+        <v>46309</v>
       </c>
     </row>
   </sheetData>
@@ -40921,10 +39981,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C3" t="n">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="4">
@@ -40934,10 +39994,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="C4" t="n">
-        <v>729</v>
+        <v>730</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Update published master datasets (2026-10-22)
</commit_message>
<xml_diff>
--- a/outputs/InnovateUK_Funding_Opportunities_Latest.xlsx
+++ b/outputs/InnovateUK_Funding_Opportunities_Latest.xlsx
@@ -1031,7 +1031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1109,26 +1109,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Innovate UK Business Connect</t>
+          <t>Innovate Funding Service</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ARIA: Standards and benchmarks for dexterous robotics</t>
+          <t>Healthy Soils and Water for a Sustainable Environment</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/aria-standards-and-benchmarks-for-dexterous-robotics/</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2604/overview/0a26a044-e3c5-4fa0-8556-b382497374df</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-21 14:43</t>
+          <t>2026-10-22 14:49</t>
         </is>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46316.61319444444</v>
+        <v>46317.61736111111</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
@@ -1137,23 +1137,19 @@
       <c r="H2" t="b">
         <v>0</v>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>19/10/2026</t>
-        </is>
-      </c>
-      <c r="J2" s="1" t="n">
-        <v>46314</v>
-      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>01/12/2026</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
+          <t>Thursday 28 January 2027 11:00am</t>
+        </is>
+      </c>
+      <c r="L2" s="1" t="n">
+        <v>46415.45833333334</v>
+      </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>£3.0 million</t>
+          <t>£5.0 million</t>
         </is>
       </c>
       <c r="N2" s="1" t="n">
@@ -1168,12 +1164,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>UK Space Agency: Unlocking Space for Business - Environmental Intelligence and Emissions</t>
+          <t>ARIA: Standards and benchmarks for dexterous robotics</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/uk-space-agency-unlocking-space-for-business-environmental-intelligence-and-emissions/</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/aria-standards-and-benchmarks-for-dexterous-robotics/</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1193,21 +1189,21 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>20/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="J3" s="1" t="n">
-        <v>46315</v>
+        <v>46314</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>11/12/2026</t>
+          <t>01/12/2026</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>£2.0 million</t>
+          <t>£3.0 million</t>
         </is>
       </c>
       <c r="N3" s="1" t="n">
@@ -1222,12 +1218,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>EIT Urban Mobility: SME Market Expansion Open Call 2027</t>
+          <t>UK Space Agency: Unlocking Space for Business - Environmental Intelligence and Emissions</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/eit-urban-mobility-sme-market-expansion-open-call-2027/</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/uk-space-agency-unlocking-space-for-business-environmental-intelligence-and-emissions/</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1247,20 +1243,74 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
+          <t>20/10/2026</t>
+        </is>
+      </c>
+      <c r="J4" s="1" t="n">
+        <v>46315</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>11/12/2026</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>£2.0 million</t>
+        </is>
+      </c>
+      <c r="N4" s="1" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Innovate UK Business Connect</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>EIT Urban Mobility: SME Market Expansion Open Call 2027</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://iuk-business-connect.org.uk/opportunities/eit-urban-mobility-sme-market-expansion-open-call-2027/</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-10-21 14:43</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>46316.61319444444</v>
+      </c>
+      <c r="F5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="b">
+        <v>0</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
           <t>09/10/2026</t>
         </is>
       </c>
-      <c r="J4" s="1" t="n">
+      <c r="J5" s="1" t="n">
         <v>46304</v>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>01/12/2026</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" s="1" t="n">
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" s="1" t="n">
         <v>46316</v>
       </c>
     </row>
@@ -1305,13 +1355,13 @@
         <v>46316</v>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C2" t="n">
         <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -2319,7 +2369,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N743"/>
+  <dimension ref="A1:N744"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -40168,6 +40218,56 @@
       <c r="M743" t="inlineStr"/>
       <c r="N743" s="1" t="n">
         <v>46309</v>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>Innovate Funding Service</t>
+        </is>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>Healthy Soils and Water for a Sustainable Environment</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2604/overview/0a26a044-e3c5-4fa0-8556-b382497374df</t>
+        </is>
+      </c>
+      <c r="D744" t="inlineStr">
+        <is>
+          <t>2026-10-22 14:49</t>
+        </is>
+      </c>
+      <c r="E744" s="1" t="n">
+        <v>46317.61736111111</v>
+      </c>
+      <c r="F744" t="b">
+        <v>1</v>
+      </c>
+      <c r="G744" t="inlineStr"/>
+      <c r="H744" t="b">
+        <v>0</v>
+      </c>
+      <c r="I744" t="inlineStr"/>
+      <c r="J744" t="inlineStr"/>
+      <c r="K744" t="inlineStr">
+        <is>
+          <t>Thursday 28 January 2027 11:00am</t>
+        </is>
+      </c>
+      <c r="L744" s="1" t="n">
+        <v>46415.45833333334</v>
+      </c>
+      <c r="M744" t="inlineStr">
+        <is>
+          <t>£5.0 million</t>
+        </is>
+      </c>
+      <c r="N744" s="1" t="n">
+        <v>46316</v>
       </c>
     </row>
   </sheetData>
@@ -40221,10 +40321,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C3" t="n">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="4">
@@ -40234,10 +40334,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="C4" t="n">
-        <v>742</v>
+        <v>743</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Update published master datasets (2026-10-26)
</commit_message>
<xml_diff>
--- a/outputs/InnovateUK_Funding_Opportunities_Latest.xlsx
+++ b/outputs/InnovateUK_Funding_Opportunities_Latest.xlsx
@@ -1031,7 +1031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1109,26 +1109,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Innovate UK Business Connect</t>
+          <t>Innovate Funding Service</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>iX Challenge: Systemic capture and analysis of structural condition data</t>
+          <t>Underground hydrogen storage demonstrator DEVEX support</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/ix-challenge-systemic-capture-and-analysis-of-structural-condition-data/</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2608/overview/edd17e49-cb74-4ae3-89ee-0ceed80c4618</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-24 13:41</t>
+          <t>2026-10-26 16:25</t>
         </is>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46319.57013888889</v>
+        <v>46321.68402777778</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
@@ -1137,21 +1137,21 @@
       <c r="H2" t="b">
         <v>0</v>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>23/10/2026</t>
-        </is>
-      </c>
-      <c r="J2" s="1" t="n">
-        <v>46318</v>
-      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>04/12/2026</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
+          <t>Wednesday 13 January 2027 11:00am</t>
+        </is>
+      </c>
+      <c r="L2" s="1" t="n">
+        <v>46400.45833333334</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>£750,000</t>
+        </is>
+      </c>
       <c r="N2" s="1" t="n">
         <v>46316</v>
       </c>
@@ -1159,26 +1159,26 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Innovate UK Business Connect</t>
+          <t>Innovate Funding Service</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Secure Innovation Security Reviews</t>
+          <t>Testing and validating underground hydrogen storage components</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/secure-innovation-security-review/</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2606/overview/52a725a1-ecfe-4eec-a30a-ac6d4078c350</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-23 14:29</t>
+          <t>2026-10-26 16:25</t>
         </is>
       </c>
       <c r="E3" s="1" t="n">
-        <v>46318.60347222222</v>
+        <v>46321.68402777778</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
@@ -1187,25 +1187,19 @@
       <c r="H3" t="b">
         <v>0</v>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>23/10/2026</t>
-        </is>
-      </c>
-      <c r="J3" s="1" t="n">
-        <v>46318</v>
-      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>31/01/2027                              12:00</t>
+          <t>Wednesday 13 January 2027 11:00am</t>
         </is>
       </c>
       <c r="L3" s="1" t="n">
-        <v>46418.5</v>
+        <v>46400.45833333334</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>£315,000</t>
+          <t>£5.0 million</t>
         </is>
       </c>
       <c r="N3" s="1" t="n">
@@ -1215,26 +1209,26 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Innovate Funding Service</t>
+          <t>Innovate UK Business Connect</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Healthy Soils and Water for a Sustainable Environment</t>
+          <t>iX Challenge: Systemic capture and analysis of structural condition data</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2604/overview/0a26a044-e3c5-4fa0-8556-b382497374df</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/ix-challenge-systemic-capture-and-analysis-of-structural-condition-data/</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-10-22 14:49</t>
+          <t>2026-10-24 13:41</t>
         </is>
       </c>
       <c r="E4" s="1" t="n">
-        <v>46317.61736111111</v>
+        <v>46319.57013888889</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
@@ -1243,21 +1237,21 @@
       <c r="H4" t="b">
         <v>0</v>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
+      <c r="J4" s="1" t="n">
+        <v>46318</v>
+      </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Thursday 28 January 2027 11:00am</t>
-        </is>
-      </c>
-      <c r="L4" s="1" t="n">
-        <v>46415.45833333334</v>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>£5.0 million</t>
-        </is>
-      </c>
+          <t>04/12/2026</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
       <c r="N4" s="1" t="n">
         <v>46316</v>
       </c>
@@ -1270,21 +1264,21 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ARIA: Standards and benchmarks for dexterous robotics</t>
+          <t>Secure Innovation Security Reviews</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/aria-standards-and-benchmarks-for-dexterous-robotics/</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/secure-innovation-security-review/</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-10-21 14:43</t>
+          <t>2026-10-23 14:29</t>
         </is>
       </c>
       <c r="E5" s="1" t="n">
-        <v>46316.61319444444</v>
+        <v>46318.60347222222</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
@@ -1295,21 +1289,23 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>23/10/2026</t>
         </is>
       </c>
       <c r="J5" s="1" t="n">
-        <v>46314</v>
+        <v>46318</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>01/12/2026</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
+          <t>31/01/2027                              12:00</t>
+        </is>
+      </c>
+      <c r="L5" s="1" t="n">
+        <v>46418.5</v>
+      </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>£3.0 million</t>
+          <t>£315,000</t>
         </is>
       </c>
       <c r="N5" s="1" t="n">
@@ -1319,26 +1315,26 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Innovate UK Business Connect</t>
+          <t>Innovate Funding Service</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>UK Space Agency: Unlocking Space for Business - Environmental Intelligence and Emissions</t>
+          <t>Healthy Soils and Water for a Sustainable Environment</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/uk-space-agency-unlocking-space-for-business-environmental-intelligence-and-emissions/</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2604/overview/0a26a044-e3c5-4fa0-8556-b382497374df</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-10-21 14:43</t>
+          <t>2026-10-22 14:49</t>
         </is>
       </c>
       <c r="E6" s="1" t="n">
-        <v>46316.61319444444</v>
+        <v>46317.61736111111</v>
       </c>
       <c r="F6" t="b">
         <v>1</v>
@@ -1347,23 +1343,19 @@
       <c r="H6" t="b">
         <v>0</v>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>20/10/2026</t>
-        </is>
-      </c>
-      <c r="J6" s="1" t="n">
-        <v>46315</v>
-      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>11/12/2026</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr"/>
+          <t>Thursday 28 January 2027 11:00am</t>
+        </is>
+      </c>
+      <c r="L6" s="1" t="n">
+        <v>46415.45833333334</v>
+      </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>£2.0 million</t>
+          <t>£5.0 million</t>
         </is>
       </c>
       <c r="N6" s="1" t="n">
@@ -1378,12 +1370,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>EIT Urban Mobility: SME Market Expansion Open Call 2027</t>
+          <t>ARIA: Standards and benchmarks for dexterous robotics</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/eit-urban-mobility-sme-market-expansion-open-call-2027/</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/aria-standards-and-benchmarks-for-dexterous-robotics/</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1403,20 +1395,128 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
+          <t>19/10/2026</t>
+        </is>
+      </c>
+      <c r="J7" s="1" t="n">
+        <v>46314</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>01/12/2026</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>£3.0 million</t>
+        </is>
+      </c>
+      <c r="N7" s="1" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Innovate UK Business Connect</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>UK Space Agency: Unlocking Space for Business - Environmental Intelligence and Emissions</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://iuk-business-connect.org.uk/opportunities/uk-space-agency-unlocking-space-for-business-environmental-intelligence-and-emissions/</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026-10-21 14:43</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>46316.61319444444</v>
+      </c>
+      <c r="F8" t="b">
+        <v>1</v>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="b">
+        <v>0</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>20/10/2026</t>
+        </is>
+      </c>
+      <c r="J8" s="1" t="n">
+        <v>46315</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>11/12/2026</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>£2.0 million</t>
+        </is>
+      </c>
+      <c r="N8" s="1" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Innovate UK Business Connect</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>EIT Urban Mobility: SME Market Expansion Open Call 2027</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://iuk-business-connect.org.uk/opportunities/eit-urban-mobility-sme-market-expansion-open-call-2027/</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026-10-21 14:43</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="n">
+        <v>46316.61319444444</v>
+      </c>
+      <c r="F9" t="b">
+        <v>1</v>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="b">
+        <v>0</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
           <t>09/10/2026</t>
         </is>
       </c>
-      <c r="J7" s="1" t="n">
+      <c r="J9" s="1" t="n">
         <v>46304</v>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>01/12/2026</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" s="1" t="n">
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" s="1" t="n">
         <v>46316</v>
       </c>
     </row>
@@ -1461,13 +1561,13 @@
         <v>46316</v>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C2" t="n">
         <v>5</v>
       </c>
       <c r="D2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3">
@@ -2475,7 +2575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N746"/>
+  <dimension ref="A1:N748"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -40479,6 +40579,106 @@
         </is>
       </c>
       <c r="N746" s="1" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>Innovate Funding Service</t>
+        </is>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>Underground hydrogen storage demonstrator DEVEX support</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2608/overview/edd17e49-cb74-4ae3-89ee-0ceed80c4618</t>
+        </is>
+      </c>
+      <c r="D747" t="inlineStr">
+        <is>
+          <t>2026-10-26 16:25</t>
+        </is>
+      </c>
+      <c r="E747" s="1" t="n">
+        <v>46321.68402777778</v>
+      </c>
+      <c r="F747" t="b">
+        <v>1</v>
+      </c>
+      <c r="G747" t="inlineStr"/>
+      <c r="H747" t="b">
+        <v>0</v>
+      </c>
+      <c r="I747" t="inlineStr"/>
+      <c r="J747" t="inlineStr"/>
+      <c r="K747" t="inlineStr">
+        <is>
+          <t>Wednesday 13 January 2027 11:00am</t>
+        </is>
+      </c>
+      <c r="L747" s="1" t="n">
+        <v>46400.45833333334</v>
+      </c>
+      <c r="M747" t="inlineStr">
+        <is>
+          <t>£750,000</t>
+        </is>
+      </c>
+      <c r="N747" s="1" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>Innovate Funding Service</t>
+        </is>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>Testing and validating underground hydrogen storage components</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2606/overview/52a725a1-ecfe-4eec-a30a-ac6d4078c350</t>
+        </is>
+      </c>
+      <c r="D748" t="inlineStr">
+        <is>
+          <t>2026-10-26 16:25</t>
+        </is>
+      </c>
+      <c r="E748" s="1" t="n">
+        <v>46321.68402777778</v>
+      </c>
+      <c r="F748" t="b">
+        <v>1</v>
+      </c>
+      <c r="G748" t="inlineStr"/>
+      <c r="H748" t="b">
+        <v>0</v>
+      </c>
+      <c r="I748" t="inlineStr"/>
+      <c r="J748" t="inlineStr"/>
+      <c r="K748" t="inlineStr">
+        <is>
+          <t>Wednesday 13 January 2027 11:00am</t>
+        </is>
+      </c>
+      <c r="L748" s="1" t="n">
+        <v>46400.45833333334</v>
+      </c>
+      <c r="M748" t="inlineStr">
+        <is>
+          <t>£5.0 million</t>
+        </is>
+      </c>
+      <c r="N748" s="1" t="n">
         <v>46316</v>
       </c>
     </row>
@@ -40533,10 +40733,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C3" t="n">
-        <v>246</v>
+        <v>248</v>
       </c>
     </row>
     <row r="4">
@@ -40546,10 +40746,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="C4" t="n">
-        <v>745</v>
+        <v>747</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Update published master datasets (2026-10-30)
</commit_message>
<xml_diff>
--- a/outputs/InnovateUK_Funding_Opportunities_Latest.xlsx
+++ b/outputs/InnovateUK_Funding_Opportunities_Latest.xlsx
@@ -1143,7 +1143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1221,26 +1221,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Innovate UK Business Connect</t>
+          <t>Innovate Funding Service</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ARIA: TA1 Integrated Robot Bodies and TA2 Foundational Technologies – Concept papers</t>
+          <t>Investor Partnerships - National Materials Innovation Programme 1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/aria-ta1-integrated-robot-bodies-and-ta2-foundational-technologies-concept-papers/</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2616/overview/d8e92206-e9dc-43d5-8d52-4fbfbd78339c</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-28 16:18</t>
+          <t>2026-10-30 16:28</t>
         </is>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46323.67916666667</v>
+        <v>46325.68611111111</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
@@ -1251,11 +1251,17 @@
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Tuesday 19 January 2027 11:00am</t>
+        </is>
+      </c>
+      <c r="L2" s="1" t="n">
+        <v>46406.45833333334</v>
+      </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>£15</t>
+          <t>£2.0 million</t>
         </is>
       </c>
       <c r="N2" s="1" t="n">
@@ -1270,12 +1276,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>EIT Higher Education Initiative Call for Proposals 2026</t>
+          <t>ARIA: TA1 Integrated Robot Bodies and TA2 Foundational Technologies – Concept papers</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/eit-higher-education-initiative-call-for-proposals-2026/</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/aria-ta1-integrated-robot-bodies-and-ta2-foundational-technologies-concept-papers/</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1293,22 +1299,66 @@
       <c r="H3" t="b">
         <v>0</v>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>£15</t>
+        </is>
+      </c>
+      <c r="N3" s="1" t="n">
+        <v>46323</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Innovate UK Business Connect</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>EIT Higher Education Initiative Call for Proposals 2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://iuk-business-connect.org.uk/opportunities/eit-higher-education-initiative-call-for-proposals-2026/</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-10-28 16:18</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>46323.67916666667</v>
+      </c>
+      <c r="F4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="b">
+        <v>0</v>
+      </c>
+      <c r="I4" t="inlineStr">
         <is>
           <t>20/10/2026</t>
         </is>
       </c>
-      <c r="J3" s="1" t="n">
+      <c r="J4" s="1" t="n">
         <v>46315</v>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>13/01/2027</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" s="1" t="n">
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" s="1" t="n">
         <v>46323</v>
       </c>
     </row>
@@ -1353,13 +1403,13 @@
         <v>46323</v>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C2" t="n">
         <v>2</v>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -2381,7 +2431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N754"/>
+  <dimension ref="A1:N755"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -40798,6 +40848,56 @@
       </c>
       <c r="N754" s="1" t="n">
         <v>46316</v>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>Innovate Funding Service</t>
+        </is>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>Investor Partnerships - National Materials Innovation Programme 1</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2616/overview/d8e92206-e9dc-43d5-8d52-4fbfbd78339c</t>
+        </is>
+      </c>
+      <c r="D755" t="inlineStr">
+        <is>
+          <t>2026-10-30 16:28</t>
+        </is>
+      </c>
+      <c r="E755" s="1" t="n">
+        <v>46325.68611111111</v>
+      </c>
+      <c r="F755" t="b">
+        <v>1</v>
+      </c>
+      <c r="G755" t="inlineStr"/>
+      <c r="H755" t="b">
+        <v>0</v>
+      </c>
+      <c r="I755" t="inlineStr"/>
+      <c r="J755" t="inlineStr"/>
+      <c r="K755" t="inlineStr">
+        <is>
+          <t>Tuesday 19 January 2027 11:00am</t>
+        </is>
+      </c>
+      <c r="L755" s="1" t="n">
+        <v>46406.45833333334</v>
+      </c>
+      <c r="M755" t="inlineStr">
+        <is>
+          <t>£2.0 million</t>
+        </is>
+      </c>
+      <c r="N755" s="1" t="n">
+        <v>46323</v>
       </c>
     </row>
   </sheetData>
@@ -40851,10 +40951,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C3" t="n">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="4">
@@ -40864,10 +40964,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="C4" t="n">
-        <v>753</v>
+        <v>754</v>
       </c>
     </row>
     <row r="5">

</xml_diff>